<commit_message>
Major upgrades — CAPM, search, constraints, 10yr returns
</commit_message>
<xml_diff>
--- a/optimised_portfolios.xlsx
+++ b/optimised_portfolios.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -470,85 +470,65 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>RELIANCE.NS</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>23.78</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>HDFCBANK.NS</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>INFY.NS</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SNOW</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>22.37</v>
-      </c>
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>13.85</v>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio Return (%)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>-9.199999999999999</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio Volatility (%)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>21.31</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Return (%)</t>
+          <t>Portfolio Sharpe Ratio</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>197.17</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Portfolio Volatility (%)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>40.43</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Portfolio Sharpe Ratio</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>4.7881</v>
+        <v>-0.737</v>
       </c>
     </row>
   </sheetData>
@@ -562,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -584,85 +564,65 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>RELIANCE.NS</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>14.34</v>
+        <v>13.48</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>HDFCBANK.NS</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>28.51</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>INFY.NS</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0</v>
+        <v>35.17</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SNOW</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>40</v>
-      </c>
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>17.15</v>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio Return (%)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>-18.7</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio Volatility (%)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>17.38</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Return (%)</t>
+          <t>Portfolio Sharpe Ratio</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>138.12</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Portfolio Volatility (%)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>37.06</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Portfolio Sharpe Ratio</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>3.6306</v>
+        <v>-1.45</v>
       </c>
     </row>
   </sheetData>
@@ -676,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -698,85 +658,65 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>RELIANCE.NS</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>HDFCBANK.NS</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>INFY.NS</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SNOW</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>20</v>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio Return (%)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>9.6</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio Volatility (%)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>19.31</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Portfolio Return (%)</t>
+          <t>Portfolio Sharpe Ratio</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>222.68</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Portfolio Volatility (%)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>47.52</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Portfolio Sharpe Ratio</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>4.6105</v>
+        <v>0.1607</v>
       </c>
     </row>
   </sheetData>

</xml_diff>